<commit_message>
Top-100 VC list: identify 7 of the 11 unreadable logos from published copies of the ranking
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2WBTUaYVg19XogRfpJJ3d
</commit_message>
<xml_diff>
--- a/collateral/SimReal-Top100VC-2026.xlsx
+++ b/collateral/SimReal-Top100VC-2026.xlsx
@@ -860,7 +860,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>待确认（logo 看不清，按代表投资推断）</t>
+          <t>已核实（f4.fund、Rothschild 均列第 14）</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -1095,7 +1095,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>（被遮挡，无法辨认）</t>
+          <t>Dragoneer Investment Group</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
@@ -1108,10 +1108,14 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr"/>
+          <t>已核实（The VC Corner 列 Dragoneer 第 23）</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>dragoneer.com</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1619,7 +1623,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>（V 字 logo，可能是 Vy Capital）</t>
+          <t>（可能是 Vy Capital）</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
@@ -1632,7 +1636,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>待确认（xAI 的第三家；logo 是 V 字，没找到排名原文）</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr"/>
@@ -1699,7 +1703,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>（无法辨认）</t>
+          <t>First Round Capital</t>
         </is>
       </c>
       <c r="C46" s="2" t="n">
@@ -1712,10 +1716,14 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr"/>
+          <t>已核实（f4.fund 列第 45；logo 是方括号）</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>firstround.com</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -1779,7 +1787,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>（可能是 Lux Capital）</t>
+          <t>Lux Capital</t>
         </is>
       </c>
       <c r="C49" s="2" t="n">
@@ -1792,10 +1800,14 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="F49" s="2" t="inlineStr"/>
+          <t>已核实（f4.fund 列第 48）</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>luxcapital.com</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -2103,7 +2115,7 @@
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>2468 Ventures（按 logo 文字）</t>
+          <t>2468 Ventures</t>
         </is>
       </c>
       <c r="C61" s="2" t="n">
@@ -2116,7 +2128,7 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>较可能（logo 文字清楚，Tracxn 显示投过 Anthropic，没找到排名原文）</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr"/>
@@ -2239,7 +2251,7 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>TeleSoft（按 logo 文字）</t>
+          <t>（可能是 IDG Capital）</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
@@ -2252,7 +2264,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>待确认（早期投资 SHEIN、红底白字 logo；没找到排名原文）</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr"/>
@@ -2315,7 +2327,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>（带翅膀的 logo，无法辨认）</t>
+          <t>（无法辨认）</t>
         </is>
       </c>
       <c r="C69" s="2" t="n">
@@ -2328,7 +2340,7 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>待确认（没查到）</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr"/>
@@ -2615,7 +2627,7 @@
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>（无法辨认）</t>
+          <t>Houston Ventures</t>
         </is>
       </c>
       <c r="C80" s="2" t="n">
@@ -2628,7 +2640,7 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>已核实（f4.fund 列第 79）</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr"/>
@@ -3063,7 +3075,7 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>（CV 开头，可能是 Curative Ventures）</t>
+          <t>Curative Ventures</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
@@ -3076,7 +3088,7 @@
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>较可能（Instil Bio 最大股东，logo 文字吻合；没找到排名原文）</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr"/>
@@ -3115,7 +3127,7 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>（圆形 logo，无法辨认）</t>
+          <t>（可能是 Innovation Endeavors）</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
@@ -3128,7 +3140,7 @@
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>待确认（领投过 AlphaSense B 轮；没找到排名原文）</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr"/>
@@ -3209,7 +3221,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>辨认把握：清楚 = logo 文字可读；较清楚 = logo 可辨但有点糊；待确认 = logo 太小或被遮挡，按代表投资推断或暂时空着。</t>
+          <t>辨认把握：清楚 = logo 文字可读；较清楚 = logo 可辨但有点糊；已核实 = 看不清的 logo 已用公开的排名转载（f4.fund、The VC Corner、Rothschild）对上；较可能 = 证据吻合但没找到排名原文；待确认 = 还没查到，括号里是最可能的候选。</t>
         </is>
       </c>
     </row>
@@ -3223,7 +3235,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SimReal-Top100VC-Apollo导入.csv 只含已辨认的机构（Company Name, Website 两列），可以在 Apollo 里用 CSV 导入批量查公司。</t>
+          <t>SimReal-Top100VC-Apollo导入.csv 收了除'待确认'以外的机构（Company Name, Website 两列），可以在 Apollo 里用 CSV 导入批量查公司；'待确认'的几家可以按括号里的候选名单独搜。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rebuild the top-100 sheet with the new stage columns (empty until research lands)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2WBTUaYVg19XogRfpJJ3d
</commit_message>
<xml_diff>
--- a/collateral/SimReal-Top100VC-2026.xlsx
+++ b/collateral/SimReal-Top100VC-2026.xlsx
@@ -11,7 +11,7 @@
     <sheet name="说明" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Top 100'!$A$1:$F$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Top 100'!$A$1:$P$101</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -434,15 +434,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:P101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="44" customWidth="1" min="14" max="14"/>
+    <col width="26" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -468,10 +478,60 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>投资阶段</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>主力阶段</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>适合我们的种子轮</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>种子项目 / 渠道</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>首笔金额</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>领投</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>方向</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>阶段信息把握</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>阶段来源</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>辨认把握</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>官网域名</t>
         </is>
@@ -494,12 +554,22 @@
           <t>DoorDash</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>sequoiacap.com</t>
         </is>
@@ -522,12 +592,22 @@
           <t>Databricks</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
         <is>
           <t>a16z.com</t>
         </is>
@@ -550,12 +630,22 @@
           <t>Scale AI</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
         <is>
           <t>accel.com</t>
         </is>
@@ -578,12 +668,22 @@
           <t>Kuaishou</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr"/>
+      <c r="N5" s="2" t="inlineStr"/>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>dst-global.com</t>
         </is>
@@ -606,12 +706,22 @@
           <t>Coinbase</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
+      <c r="N6" s="2" t="inlineStr"/>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
         <is>
           <t>tigerglobal.com</t>
         </is>
@@ -634,12 +744,22 @@
           <t>Figma</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="inlineStr"/>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
         <is>
           <t>indexventures.com</t>
         </is>
@@ -662,12 +782,22 @@
           <t>Mistral AI</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr"/>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
         <is>
           <t>lsvp.com</t>
         </is>
@@ -690,12 +820,22 @@
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr"/>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
         <is>
           <t>thrivecap.com</t>
         </is>
@@ -718,12 +858,22 @@
           <t>Ramp</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
         <is>
           <t>foundersfund.com</t>
         </is>
@@ -746,12 +896,22 @@
           <t>Snowflake</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
         <is>
           <t>iconiqcapital.com</t>
         </is>
@@ -774,12 +934,22 @@
           <t>Figma</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
         <is>
           <t>kleinerperkins.com</t>
         </is>
@@ -802,12 +972,22 @@
           <t>Robinhood</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr"/>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
         <is>
           <t>nea.com</t>
         </is>
@@ -830,12 +1010,22 @@
           <t>Figma</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr"/>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
         <is>
           <t>greylock.com</t>
         </is>
@@ -858,12 +1048,22 @@
           <t>Sierra</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr"/>
+      <c r="O15" s="2" t="inlineStr">
         <is>
           <t>已核实（f4.fund、Rothschild 均列第 14）</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="P15" s="2" t="inlineStr">
         <is>
           <t>benchmark.com</t>
         </is>
@@ -886,12 +1086,22 @@
           <t>Perplexity</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr"/>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
         <is>
           <t>bvp.com</t>
         </is>
@@ -914,12 +1124,22 @@
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr"/>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
         <is>
           <t>khoslaventures.com</t>
         </is>
@@ -942,12 +1162,22 @@
           <t>Athelas</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr"/>
+      <c r="N18" s="2" t="inlineStr"/>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
         <is>
           <t>generalcatalyst.com</t>
         </is>
@@ -970,12 +1200,22 @@
           <t>Robinhood</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="inlineStr"/>
+      <c r="N19" s="2" t="inlineStr"/>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
         <is>
           <t>ribbitcap.com</t>
         </is>
@@ -998,12 +1238,22 @@
           <t>Figure</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
+      <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr"/>
+      <c r="N20" s="2" t="inlineStr"/>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1022,12 +1272,22 @@
           <t>ByteDance</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr"/>
+      <c r="N21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
         <is>
           <t>generalatlantic.com</t>
         </is>
@@ -1050,12 +1310,22 @@
           <t>HashiCorp</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr"/>
+      <c r="M22" s="2" t="inlineStr"/>
+      <c r="N22" s="2" t="inlineStr"/>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
         <is>
           <t>notablecap.com</t>
         </is>
@@ -1078,12 +1348,22 @@
           <t>Perplexity</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="inlineStr"/>
+      <c r="M23" s="2" t="inlineStr"/>
+      <c r="N23" s="2" t="inlineStr"/>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
         <is>
           <t>ivp.com</t>
         </is>
@@ -1106,12 +1386,22 @@
           <t>Klarna</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="inlineStr"/>
+      <c r="N24" s="2" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr">
         <is>
           <t>已核实（The VC Corner 列 Dragoneer 第 23）</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="P24" s="2" t="inlineStr">
         <is>
           <t>dragoneer.com</t>
         </is>
@@ -1134,12 +1424,22 @@
           <t>Snowflake</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr"/>
+      <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr"/>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr"/>
+      <c r="M25" s="2" t="inlineStr"/>
+      <c r="N25" s="2" t="inlineStr"/>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
         <is>
           <t>altimeter.com</t>
         </is>
@@ -1162,12 +1462,22 @@
           <t>HashiCorp</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr"/>
+      <c r="N26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
         <is>
           <t>mayfield.com</t>
         </is>
@@ -1190,12 +1500,22 @@
           <t>Snowflake</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr"/>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr"/>
+      <c r="M27" s="2" t="inlineStr"/>
+      <c r="N27" s="2" t="inlineStr"/>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
         <is>
           <t>shv.com</t>
         </is>
@@ -1218,12 +1538,22 @@
           <t>AbCellera</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr"/>
+      <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr"/>
+      <c r="M28" s="2" t="inlineStr"/>
+      <c r="N28" s="2" t="inlineStr"/>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
         <is>
           <t>orbimed.com</t>
         </is>
@@ -1246,12 +1576,22 @@
           <t>Checkout.com</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr"/>
+      <c r="J29" s="2" t="inlineStr"/>
+      <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="inlineStr"/>
+      <c r="N29" s="2" t="inlineStr"/>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
         <is>
           <t>insightpartners.com</t>
         </is>
@@ -1274,12 +1614,22 @@
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr"/>
+      <c r="J30" s="2" t="inlineStr"/>
+      <c r="K30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr"/>
+      <c r="M30" s="2" t="inlineStr"/>
+      <c r="N30" s="2" t="inlineStr"/>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
         <is>
           <t>coatue.com</t>
         </is>
@@ -1302,12 +1652,22 @@
           <t>Perch</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr"/>
+      <c r="F31" s="2" t="inlineStr"/>
+      <c r="G31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="inlineStr"/>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr"/>
+      <c r="L31" s="2" t="inlineStr"/>
+      <c r="M31" s="2" t="inlineStr"/>
+      <c r="N31" s="2" t="inlineStr"/>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="inlineStr">
         <is>
           <t>sparkcapital.com</t>
         </is>
@@ -1330,12 +1690,22 @@
           <t>Sierra</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr"/>
+      <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr"/>
+      <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr"/>
+      <c r="L32" s="2" t="inlineStr"/>
+      <c r="M32" s="2" t="inlineStr"/>
+      <c r="N32" s="2" t="inlineStr"/>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
         <is>
           <t>svangel.com</t>
         </is>
@@ -1358,12 +1728,22 @@
           <t>Braze</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="E33" s="2" t="inlineStr"/>
+      <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr"/>
+      <c r="L33" s="2" t="inlineStr"/>
+      <c r="M33" s="2" t="inlineStr"/>
+      <c r="N33" s="2" t="inlineStr"/>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="inlineStr">
         <is>
           <t>battery.com</t>
         </is>
@@ -1386,12 +1766,22 @@
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
+      <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr"/>
+      <c r="J34" s="2" t="inlineStr"/>
+      <c r="K34" s="2" t="inlineStr"/>
+      <c r="L34" s="2" t="inlineStr"/>
+      <c r="M34" s="2" t="inlineStr"/>
+      <c r="N34" s="2" t="inlineStr"/>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -1410,12 +1800,22 @@
           <t>Fireblocks</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr"/>
+      <c r="K35" s="2" t="inlineStr"/>
+      <c r="L35" s="2" t="inlineStr"/>
+      <c r="M35" s="2" t="inlineStr"/>
+      <c r="N35" s="2" t="inlineStr"/>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P35" s="2" t="inlineStr">
         <is>
           <t>paradigm.xyz</t>
         </is>
@@ -1438,12 +1838,22 @@
           <t>CareBridge（看不清）</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr"/>
+      <c r="G36" s="2" t="inlineStr"/>
+      <c r="H36" s="2" t="inlineStr"/>
+      <c r="I36" s="2" t="inlineStr"/>
+      <c r="J36" s="2" t="inlineStr"/>
+      <c r="K36" s="2" t="inlineStr"/>
+      <c r="L36" s="2" t="inlineStr"/>
+      <c r="M36" s="2" t="inlineStr"/>
+      <c r="N36" s="2" t="inlineStr"/>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P36" s="2" t="inlineStr">
         <is>
           <t>oakhcft.com</t>
         </is>
@@ -1466,12 +1876,22 @@
           <t>Akero Therapeutics</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr"/>
+      <c r="F37" s="2" t="inlineStr"/>
+      <c r="G37" s="2" t="inlineStr"/>
+      <c r="H37" s="2" t="inlineStr"/>
+      <c r="I37" s="2" t="inlineStr"/>
+      <c r="J37" s="2" t="inlineStr"/>
+      <c r="K37" s="2" t="inlineStr"/>
+      <c r="L37" s="2" t="inlineStr"/>
+      <c r="M37" s="2" t="inlineStr"/>
+      <c r="N37" s="2" t="inlineStr"/>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P37" s="2" t="inlineStr">
         <is>
           <t>atlasventure.com</t>
         </is>
@@ -1494,12 +1914,22 @@
           <t>Devoted Health</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr"/>
+      <c r="G38" s="2" t="inlineStr"/>
+      <c r="H38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr"/>
+      <c r="J38" s="2" t="inlineStr"/>
+      <c r="K38" s="2" t="inlineStr"/>
+      <c r="L38" s="2" t="inlineStr"/>
+      <c r="M38" s="2" t="inlineStr"/>
+      <c r="N38" s="2" t="inlineStr"/>
+      <c r="O38" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P38" s="2" t="inlineStr">
         <is>
           <t>venrock.com</t>
         </is>
@@ -1522,12 +1952,22 @@
           <t>Flock Safety</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr"/>
+      <c r="F39" s="2" t="inlineStr"/>
+      <c r="G39" s="2" t="inlineStr"/>
+      <c r="H39" s="2" t="inlineStr"/>
+      <c r="I39" s="2" t="inlineStr"/>
+      <c r="J39" s="2" t="inlineStr"/>
+      <c r="K39" s="2" t="inlineStr"/>
+      <c r="L39" s="2" t="inlineStr"/>
+      <c r="M39" s="2" t="inlineStr"/>
+      <c r="N39" s="2" t="inlineStr"/>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P39" s="2" t="inlineStr">
         <is>
           <t>meritechcapital.com</t>
         </is>
@@ -1550,12 +1990,22 @@
           <t>Vast</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr"/>
+      <c r="G40" s="2" t="inlineStr"/>
+      <c r="H40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr"/>
+      <c r="J40" s="2" t="inlineStr"/>
+      <c r="K40" s="2" t="inlineStr"/>
+      <c r="L40" s="2" t="inlineStr"/>
+      <c r="M40" s="2" t="inlineStr"/>
+      <c r="N40" s="2" t="inlineStr"/>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P40" s="2" t="inlineStr">
         <is>
           <t>nvp.com</t>
         </is>
@@ -1578,12 +2028,22 @@
           <t>Reflection AI</t>
         </is>
       </c>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr"/>
+      <c r="F41" s="2" t="inlineStr"/>
+      <c r="G41" s="2" t="inlineStr"/>
+      <c r="H41" s="2" t="inlineStr"/>
+      <c r="I41" s="2" t="inlineStr"/>
+      <c r="J41" s="2" t="inlineStr"/>
+      <c r="K41" s="2" t="inlineStr"/>
+      <c r="L41" s="2" t="inlineStr"/>
+      <c r="M41" s="2" t="inlineStr"/>
+      <c r="N41" s="2" t="inlineStr"/>
+      <c r="O41" s="2" t="inlineStr">
         <is>
           <t>较清楚（红色圆形 logo）</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr">
+      <c r="P41" s="2" t="inlineStr">
         <is>
           <t>crv.com</t>
         </is>
@@ -1606,12 +2066,22 @@
           <t>Crusoe</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr"/>
+      <c r="G42" s="2" t="inlineStr"/>
+      <c r="H42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr"/>
+      <c r="L42" s="2" t="inlineStr"/>
+      <c r="M42" s="2" t="inlineStr"/>
+      <c r="N42" s="2" t="inlineStr"/>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="inlineStr">
         <is>
           <t>baincapitalventures.com</t>
         </is>
@@ -1634,12 +2104,22 @@
           <t>xAI</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="E43" s="2" t="inlineStr"/>
+      <c r="F43" s="2" t="inlineStr"/>
+      <c r="G43" s="2" t="inlineStr"/>
+      <c r="H43" s="2" t="inlineStr"/>
+      <c r="I43" s="2" t="inlineStr"/>
+      <c r="J43" s="2" t="inlineStr"/>
+      <c r="K43" s="2" t="inlineStr"/>
+      <c r="L43" s="2" t="inlineStr"/>
+      <c r="M43" s="2" t="inlineStr"/>
+      <c r="N43" s="2" t="inlineStr"/>
+      <c r="O43" s="2" t="inlineStr">
         <is>
           <t>待确认（xAI 的第三家；logo 是 V 字，没找到排名原文）</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr"/>
+      <c r="P43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -1658,12 +2138,22 @@
           <t>Anthropic</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr"/>
+      <c r="G44" s="2" t="inlineStr"/>
+      <c r="H44" s="2" t="inlineStr"/>
+      <c r="I44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr"/>
+      <c r="K44" s="2" t="inlineStr"/>
+      <c r="L44" s="2" t="inlineStr"/>
+      <c r="M44" s="2" t="inlineStr"/>
+      <c r="N44" s="2" t="inlineStr"/>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P44" s="2" t="inlineStr">
         <is>
           <t>menlovc.com</t>
         </is>
@@ -1686,12 +2176,22 @@
           <t>Coupang</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F45" s="2" t="inlineStr">
+      <c r="E45" s="2" t="inlineStr"/>
+      <c r="F45" s="2" t="inlineStr"/>
+      <c r="G45" s="2" t="inlineStr"/>
+      <c r="H45" s="2" t="inlineStr"/>
+      <c r="I45" s="2" t="inlineStr"/>
+      <c r="J45" s="2" t="inlineStr"/>
+      <c r="K45" s="2" t="inlineStr"/>
+      <c r="L45" s="2" t="inlineStr"/>
+      <c r="M45" s="2" t="inlineStr"/>
+      <c r="N45" s="2" t="inlineStr"/>
+      <c r="O45" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P45" s="2" t="inlineStr">
         <is>
           <t>greenoaks.com</t>
         </is>
@@ -1714,12 +2214,22 @@
           <t>Verkada</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr"/>
+      <c r="G46" s="2" t="inlineStr"/>
+      <c r="H46" s="2" t="inlineStr"/>
+      <c r="I46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr"/>
+      <c r="K46" s="2" t="inlineStr"/>
+      <c r="L46" s="2" t="inlineStr"/>
+      <c r="M46" s="2" t="inlineStr"/>
+      <c r="N46" s="2" t="inlineStr"/>
+      <c r="O46" s="2" t="inlineStr">
         <is>
           <t>已核实（f4.fund 列第 45；logo 是方括号）</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="P46" s="2" t="inlineStr">
         <is>
           <t>firstround.com</t>
         </is>
@@ -1742,12 +2252,22 @@
           <t>Chaos Industries</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr">
+      <c r="E47" s="2" t="inlineStr"/>
+      <c r="F47" s="2" t="inlineStr"/>
+      <c r="G47" s="2" t="inlineStr"/>
+      <c r="H47" s="2" t="inlineStr"/>
+      <c r="I47" s="2" t="inlineStr"/>
+      <c r="J47" s="2" t="inlineStr"/>
+      <c r="K47" s="2" t="inlineStr"/>
+      <c r="L47" s="2" t="inlineStr"/>
+      <c r="M47" s="2" t="inlineStr"/>
+      <c r="N47" s="2" t="inlineStr"/>
+      <c r="O47" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P47" s="2" t="inlineStr">
         <is>
           <t>8vc.com</t>
         </is>
@@ -1770,12 +2290,22 @@
           <t>Toast</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr"/>
+      <c r="G48" s="2" t="inlineStr"/>
+      <c r="H48" s="2" t="inlineStr"/>
+      <c r="I48" s="2" t="inlineStr"/>
+      <c r="J48" s="2" t="inlineStr"/>
+      <c r="K48" s="2" t="inlineStr"/>
+      <c r="L48" s="2" t="inlineStr"/>
+      <c r="M48" s="2" t="inlineStr"/>
+      <c r="N48" s="2" t="inlineStr"/>
+      <c r="O48" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P48" s="2" t="inlineStr">
         <is>
           <t>tcv.com</t>
         </is>
@@ -1798,12 +2328,22 @@
           <t>Ramp</t>
         </is>
       </c>
-      <c r="E49" s="2" t="inlineStr">
+      <c r="E49" s="2" t="inlineStr"/>
+      <c r="F49" s="2" t="inlineStr"/>
+      <c r="G49" s="2" t="inlineStr"/>
+      <c r="H49" s="2" t="inlineStr"/>
+      <c r="I49" s="2" t="inlineStr"/>
+      <c r="J49" s="2" t="inlineStr"/>
+      <c r="K49" s="2" t="inlineStr"/>
+      <c r="L49" s="2" t="inlineStr"/>
+      <c r="M49" s="2" t="inlineStr"/>
+      <c r="N49" s="2" t="inlineStr"/>
+      <c r="O49" s="2" t="inlineStr">
         <is>
           <t>已核实（f4.fund 列第 48）</t>
         </is>
       </c>
-      <c r="F49" s="2" t="inlineStr">
+      <c r="P49" s="2" t="inlineStr">
         <is>
           <t>luxcapital.com</t>
         </is>
@@ -1826,12 +2366,22 @@
           <t>Sana Biotechnology</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr"/>
+      <c r="G50" s="2" t="inlineStr"/>
+      <c r="H50" s="2" t="inlineStr"/>
+      <c r="I50" s="2" t="inlineStr"/>
+      <c r="J50" s="2" t="inlineStr"/>
+      <c r="K50" s="2" t="inlineStr"/>
+      <c r="L50" s="2" t="inlineStr"/>
+      <c r="M50" s="2" t="inlineStr"/>
+      <c r="N50" s="2" t="inlineStr"/>
+      <c r="O50" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P50" s="2" t="inlineStr">
         <is>
           <t>archventure.com</t>
         </is>
@@ -1854,12 +2404,22 @@
           <t>Coinbase</t>
         </is>
       </c>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F51" s="2" t="inlineStr">
+      <c r="E51" s="2" t="inlineStr"/>
+      <c r="F51" s="2" t="inlineStr"/>
+      <c r="G51" s="2" t="inlineStr"/>
+      <c r="H51" s="2" t="inlineStr"/>
+      <c r="I51" s="2" t="inlineStr"/>
+      <c r="J51" s="2" t="inlineStr"/>
+      <c r="K51" s="2" t="inlineStr"/>
+      <c r="L51" s="2" t="inlineStr"/>
+      <c r="M51" s="2" t="inlineStr"/>
+      <c r="N51" s="2" t="inlineStr"/>
+      <c r="O51" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P51" s="2" t="inlineStr">
         <is>
           <t>usv.com</t>
         </is>
@@ -1882,12 +2442,22 @@
           <t>Fivetran</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F52" s="2" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr"/>
+      <c r="F52" s="2" t="inlineStr"/>
+      <c r="G52" s="2" t="inlineStr"/>
+      <c r="H52" s="2" t="inlineStr"/>
+      <c r="I52" s="2" t="inlineStr"/>
+      <c r="J52" s="2" t="inlineStr"/>
+      <c r="K52" s="2" t="inlineStr"/>
+      <c r="L52" s="2" t="inlineStr"/>
+      <c r="M52" s="2" t="inlineStr"/>
+      <c r="N52" s="2" t="inlineStr"/>
+      <c r="O52" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P52" s="2" t="inlineStr">
         <is>
           <t>matrix.vc</t>
         </is>
@@ -1910,12 +2480,22 @@
           <t>xAI</t>
         </is>
       </c>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
+      <c r="E53" s="2" t="inlineStr"/>
       <c r="F53" s="2" t="inlineStr"/>
+      <c r="G53" s="2" t="inlineStr"/>
+      <c r="H53" s="2" t="inlineStr"/>
+      <c r="I53" s="2" t="inlineStr"/>
+      <c r="J53" s="2" t="inlineStr"/>
+      <c r="K53" s="2" t="inlineStr"/>
+      <c r="L53" s="2" t="inlineStr"/>
+      <c r="M53" s="2" t="inlineStr"/>
+      <c r="N53" s="2" t="inlineStr"/>
+      <c r="O53" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -1934,12 +2514,22 @@
           <t>Auth0</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F54" s="2" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr"/>
+      <c r="F54" s="2" t="inlineStr"/>
+      <c r="G54" s="2" t="inlineStr"/>
+      <c r="H54" s="2" t="inlineStr"/>
+      <c r="I54" s="2" t="inlineStr"/>
+      <c r="J54" s="2" t="inlineStr"/>
+      <c r="K54" s="2" t="inlineStr"/>
+      <c r="L54" s="2" t="inlineStr"/>
+      <c r="M54" s="2" t="inlineStr"/>
+      <c r="N54" s="2" t="inlineStr"/>
+      <c r="O54" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P54" s="2" t="inlineStr">
         <is>
           <t>sapphireventures.com</t>
         </is>
@@ -1962,12 +2552,22 @@
           <t>Anduril</t>
         </is>
       </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F55" s="2" t="inlineStr">
+      <c r="E55" s="2" t="inlineStr"/>
+      <c r="F55" s="2" t="inlineStr"/>
+      <c r="G55" s="2" t="inlineStr"/>
+      <c r="H55" s="2" t="inlineStr"/>
+      <c r="I55" s="2" t="inlineStr"/>
+      <c r="J55" s="2" t="inlineStr"/>
+      <c r="K55" s="2" t="inlineStr"/>
+      <c r="L55" s="2" t="inlineStr"/>
+      <c r="M55" s="2" t="inlineStr"/>
+      <c r="N55" s="2" t="inlineStr"/>
+      <c r="O55" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P55" s="2" t="inlineStr">
         <is>
           <t>valorep.com</t>
         </is>
@@ -1990,12 +2590,22 @@
           <t>Inari Medical</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr"/>
+      <c r="F56" s="2" t="inlineStr"/>
+      <c r="G56" s="2" t="inlineStr"/>
+      <c r="H56" s="2" t="inlineStr"/>
+      <c r="I56" s="2" t="inlineStr"/>
+      <c r="J56" s="2" t="inlineStr"/>
+      <c r="K56" s="2" t="inlineStr"/>
+      <c r="L56" s="2" t="inlineStr"/>
+      <c r="M56" s="2" t="inlineStr"/>
+      <c r="N56" s="2" t="inlineStr"/>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P56" s="2" t="inlineStr">
         <is>
           <t>usvp.com</t>
         </is>
@@ -2018,12 +2628,22 @@
           <t>Groq</t>
         </is>
       </c>
-      <c r="E57" s="2" t="inlineStr">
+      <c r="E57" s="2" t="inlineStr"/>
+      <c r="F57" s="2" t="inlineStr"/>
+      <c r="G57" s="2" t="inlineStr"/>
+      <c r="H57" s="2" t="inlineStr"/>
+      <c r="I57" s="2" t="inlineStr"/>
+      <c r="J57" s="2" t="inlineStr"/>
+      <c r="K57" s="2" t="inlineStr"/>
+      <c r="L57" s="2" t="inlineStr"/>
+      <c r="M57" s="2" t="inlineStr"/>
+      <c r="N57" s="2" t="inlineStr"/>
+      <c r="O57" s="2" t="inlineStr">
         <is>
           <t>较清楚</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr"/>
+      <c r="P57" s="2" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -2042,12 +2662,22 @@
           <t>xAI</t>
         </is>
       </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F58" s="2" t="inlineStr">
+      <c r="E58" s="2" t="inlineStr"/>
+      <c r="F58" s="2" t="inlineStr"/>
+      <c r="G58" s="2" t="inlineStr"/>
+      <c r="H58" s="2" t="inlineStr"/>
+      <c r="I58" s="2" t="inlineStr"/>
+      <c r="J58" s="2" t="inlineStr"/>
+      <c r="K58" s="2" t="inlineStr"/>
+      <c r="L58" s="2" t="inlineStr"/>
+      <c r="M58" s="2" t="inlineStr"/>
+      <c r="N58" s="2" t="inlineStr"/>
+      <c r="O58" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P58" s="2" t="inlineStr">
         <is>
           <t>future.ventures</t>
         </is>
@@ -2070,12 +2700,22 @@
           <t>Snowflake</t>
         </is>
       </c>
-      <c r="E59" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F59" s="2" t="inlineStr">
+      <c r="E59" s="2" t="inlineStr"/>
+      <c r="F59" s="2" t="inlineStr"/>
+      <c r="G59" s="2" t="inlineStr"/>
+      <c r="H59" s="2" t="inlineStr"/>
+      <c r="I59" s="2" t="inlineStr"/>
+      <c r="J59" s="2" t="inlineStr"/>
+      <c r="K59" s="2" t="inlineStr"/>
+      <c r="L59" s="2" t="inlineStr"/>
+      <c r="M59" s="2" t="inlineStr"/>
+      <c r="N59" s="2" t="inlineStr"/>
+      <c r="O59" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P59" s="2" t="inlineStr">
         <is>
           <t>madrona.com</t>
         </is>
@@ -2098,12 +2738,22 @@
           <t>Runway</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr">
+      <c r="E60" s="2" t="inlineStr"/>
+      <c r="F60" s="2" t="inlineStr"/>
+      <c r="G60" s="2" t="inlineStr"/>
+      <c r="H60" s="2" t="inlineStr"/>
+      <c r="I60" s="2" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr"/>
+      <c r="K60" s="2" t="inlineStr"/>
+      <c r="L60" s="2" t="inlineStr"/>
+      <c r="M60" s="2" t="inlineStr"/>
+      <c r="N60" s="2" t="inlineStr"/>
+      <c r="O60" s="2" t="inlineStr">
         <is>
           <t>较清楚</t>
         </is>
       </c>
-      <c r="F60" s="2" t="inlineStr">
+      <c r="P60" s="2" t="inlineStr">
         <is>
           <t>amplifypartners.com</t>
         </is>
@@ -2126,12 +2776,22 @@
           <t>Anthropic</t>
         </is>
       </c>
-      <c r="E61" s="2" t="inlineStr">
+      <c r="E61" s="2" t="inlineStr"/>
+      <c r="F61" s="2" t="inlineStr"/>
+      <c r="G61" s="2" t="inlineStr"/>
+      <c r="H61" s="2" t="inlineStr"/>
+      <c r="I61" s="2" t="inlineStr"/>
+      <c r="J61" s="2" t="inlineStr"/>
+      <c r="K61" s="2" t="inlineStr"/>
+      <c r="L61" s="2" t="inlineStr"/>
+      <c r="M61" s="2" t="inlineStr"/>
+      <c r="N61" s="2" t="inlineStr"/>
+      <c r="O61" s="2" t="inlineStr">
         <is>
           <t>较可能（logo 文字清楚，Tracxn 显示投过 Anthropic，没找到排名原文）</t>
         </is>
       </c>
-      <c r="F61" s="2" t="inlineStr"/>
+      <c r="P61" s="2" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -2150,12 +2810,22 @@
           <t>RayzeBio</t>
         </is>
       </c>
-      <c r="E62" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F62" s="2" t="inlineStr">
+      <c r="E62" s="2" t="inlineStr"/>
+      <c r="F62" s="2" t="inlineStr"/>
+      <c r="G62" s="2" t="inlineStr"/>
+      <c r="H62" s="2" t="inlineStr"/>
+      <c r="I62" s="2" t="inlineStr"/>
+      <c r="J62" s="2" t="inlineStr"/>
+      <c r="K62" s="2" t="inlineStr"/>
+      <c r="L62" s="2" t="inlineStr"/>
+      <c r="M62" s="2" t="inlineStr"/>
+      <c r="N62" s="2" t="inlineStr"/>
+      <c r="O62" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P62" s="2" t="inlineStr">
         <is>
           <t>versantventures.com</t>
         </is>
@@ -2178,12 +2848,22 @@
           <t>Sportradar</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F63" s="2" t="inlineStr">
+      <c r="E63" s="2" t="inlineStr"/>
+      <c r="F63" s="2" t="inlineStr"/>
+      <c r="G63" s="2" t="inlineStr"/>
+      <c r="H63" s="2" t="inlineStr"/>
+      <c r="I63" s="2" t="inlineStr"/>
+      <c r="J63" s="2" t="inlineStr"/>
+      <c r="K63" s="2" t="inlineStr"/>
+      <c r="L63" s="2" t="inlineStr"/>
+      <c r="M63" s="2" t="inlineStr"/>
+      <c r="N63" s="2" t="inlineStr"/>
+      <c r="O63" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P63" s="2" t="inlineStr">
         <is>
           <t>revolution.com</t>
         </is>
@@ -2206,12 +2886,22 @@
           <t>Peloton</t>
         </is>
       </c>
-      <c r="E64" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F64" s="2" t="inlineStr">
+      <c r="E64" s="2" t="inlineStr"/>
+      <c r="F64" s="2" t="inlineStr"/>
+      <c r="G64" s="2" t="inlineStr"/>
+      <c r="H64" s="2" t="inlineStr"/>
+      <c r="I64" s="2" t="inlineStr"/>
+      <c r="J64" s="2" t="inlineStr"/>
+      <c r="K64" s="2" t="inlineStr"/>
+      <c r="L64" s="2" t="inlineStr"/>
+      <c r="M64" s="2" t="inlineStr"/>
+      <c r="N64" s="2" t="inlineStr"/>
+      <c r="O64" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P64" s="2" t="inlineStr">
         <is>
           <t>trueventures.com</t>
         </is>
@@ -2234,12 +2924,22 @@
           <t>Alchemy</t>
         </is>
       </c>
-      <c r="E65" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F65" s="2" t="inlineStr">
+      <c r="E65" s="2" t="inlineStr"/>
+      <c r="F65" s="2" t="inlineStr"/>
+      <c r="G65" s="2" t="inlineStr"/>
+      <c r="H65" s="2" t="inlineStr"/>
+      <c r="I65" s="2" t="inlineStr"/>
+      <c r="J65" s="2" t="inlineStr"/>
+      <c r="K65" s="2" t="inlineStr"/>
+      <c r="L65" s="2" t="inlineStr"/>
+      <c r="M65" s="2" t="inlineStr"/>
+      <c r="N65" s="2" t="inlineStr"/>
+      <c r="O65" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P65" s="2" t="inlineStr">
         <is>
           <t>addition.com</t>
         </is>
@@ -2262,12 +2962,22 @@
           <t>SHEIN</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr">
+      <c r="E66" s="2" t="inlineStr"/>
+      <c r="F66" s="2" t="inlineStr"/>
+      <c r="G66" s="2" t="inlineStr"/>
+      <c r="H66" s="2" t="inlineStr"/>
+      <c r="I66" s="2" t="inlineStr"/>
+      <c r="J66" s="2" t="inlineStr"/>
+      <c r="K66" s="2" t="inlineStr"/>
+      <c r="L66" s="2" t="inlineStr"/>
+      <c r="M66" s="2" t="inlineStr"/>
+      <c r="N66" s="2" t="inlineStr"/>
+      <c r="O66" s="2" t="inlineStr">
         <is>
           <t>待确认（早期投资 SHEIN、红底白字 logo；没找到排名原文）</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr"/>
+      <c r="P66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -2286,12 +2996,22 @@
           <t>Saronic</t>
         </is>
       </c>
-      <c r="E67" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
+      <c r="E67" s="2" t="inlineStr"/>
       <c r="F67" s="2" t="inlineStr"/>
+      <c r="G67" s="2" t="inlineStr"/>
+      <c r="H67" s="2" t="inlineStr"/>
+      <c r="I67" s="2" t="inlineStr"/>
+      <c r="J67" s="2" t="inlineStr"/>
+      <c r="K67" s="2" t="inlineStr"/>
+      <c r="L67" s="2" t="inlineStr"/>
+      <c r="M67" s="2" t="inlineStr"/>
+      <c r="N67" s="2" t="inlineStr"/>
+      <c r="O67" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P67" s="2" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -2310,12 +3030,22 @@
           <t>CoreWeave</t>
         </is>
       </c>
-      <c r="E68" s="2" t="inlineStr">
+      <c r="E68" s="2" t="inlineStr"/>
+      <c r="F68" s="2" t="inlineStr"/>
+      <c r="G68" s="2" t="inlineStr"/>
+      <c r="H68" s="2" t="inlineStr"/>
+      <c r="I68" s="2" t="inlineStr"/>
+      <c r="J68" s="2" t="inlineStr"/>
+      <c r="K68" s="2" t="inlineStr"/>
+      <c r="L68" s="2" t="inlineStr"/>
+      <c r="M68" s="2" t="inlineStr"/>
+      <c r="N68" s="2" t="inlineStr"/>
+      <c r="O68" s="2" t="inlineStr">
         <is>
           <t>较清楚</t>
         </is>
       </c>
-      <c r="F68" s="2" t="inlineStr">
+      <c r="P68" s="2" t="inlineStr">
         <is>
           <t>dcvc.com</t>
         </is>
@@ -2338,12 +3068,22 @@
           <t>W 开头的公司（看不清）</t>
         </is>
       </c>
-      <c r="E69" s="2" t="inlineStr">
+      <c r="E69" s="2" t="inlineStr"/>
+      <c r="F69" s="2" t="inlineStr"/>
+      <c r="G69" s="2" t="inlineStr"/>
+      <c r="H69" s="2" t="inlineStr"/>
+      <c r="I69" s="2" t="inlineStr"/>
+      <c r="J69" s="2" t="inlineStr"/>
+      <c r="K69" s="2" t="inlineStr"/>
+      <c r="L69" s="2" t="inlineStr"/>
+      <c r="M69" s="2" t="inlineStr"/>
+      <c r="N69" s="2" t="inlineStr"/>
+      <c r="O69" s="2" t="inlineStr">
         <is>
           <t>待确认（没查到）</t>
         </is>
       </c>
-      <c r="F69" s="2" t="inlineStr"/>
+      <c r="P69" s="2" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
@@ -2362,12 +3102,22 @@
           <t>Ro</t>
         </is>
       </c>
-      <c r="E70" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F70" s="2" t="inlineStr">
+      <c r="E70" s="2" t="inlineStr"/>
+      <c r="F70" s="2" t="inlineStr"/>
+      <c r="G70" s="2" t="inlineStr"/>
+      <c r="H70" s="2" t="inlineStr"/>
+      <c r="I70" s="2" t="inlineStr"/>
+      <c r="J70" s="2" t="inlineStr"/>
+      <c r="K70" s="2" t="inlineStr"/>
+      <c r="L70" s="2" t="inlineStr"/>
+      <c r="M70" s="2" t="inlineStr"/>
+      <c r="N70" s="2" t="inlineStr"/>
+      <c r="O70" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P70" s="2" t="inlineStr">
         <is>
           <t>firstmark.com</t>
         </is>
@@ -2390,12 +3140,22 @@
           <t>FalconX</t>
         </is>
       </c>
-      <c r="E71" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F71" s="2" t="inlineStr">
+      <c r="E71" s="2" t="inlineStr"/>
+      <c r="F71" s="2" t="inlineStr"/>
+      <c r="G71" s="2" t="inlineStr"/>
+      <c r="H71" s="2" t="inlineStr"/>
+      <c r="I71" s="2" t="inlineStr"/>
+      <c r="J71" s="2" t="inlineStr"/>
+      <c r="K71" s="2" t="inlineStr"/>
+      <c r="L71" s="2" t="inlineStr"/>
+      <c r="M71" s="2" t="inlineStr"/>
+      <c r="N71" s="2" t="inlineStr"/>
+      <c r="O71" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P71" s="2" t="inlineStr">
         <is>
           <t>flybridge.com</t>
         </is>
@@ -2418,12 +3178,22 @@
           <t>Relativity</t>
         </is>
       </c>
-      <c r="E72" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F72" s="2" t="inlineStr">
+      <c r="E72" s="2" t="inlineStr"/>
+      <c r="F72" s="2" t="inlineStr"/>
+      <c r="G72" s="2" t="inlineStr"/>
+      <c r="H72" s="2" t="inlineStr"/>
+      <c r="I72" s="2" t="inlineStr"/>
+      <c r="J72" s="2" t="inlineStr"/>
+      <c r="K72" s="2" t="inlineStr"/>
+      <c r="L72" s="2" t="inlineStr"/>
+      <c r="M72" s="2" t="inlineStr"/>
+      <c r="N72" s="2" t="inlineStr"/>
+      <c r="O72" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P72" s="2" t="inlineStr">
         <is>
           <t>playground.global</t>
         </is>
@@ -2446,12 +3216,22 @@
           <t>Bobbie</t>
         </is>
       </c>
-      <c r="E73" s="2" t="inlineStr">
+      <c r="E73" s="2" t="inlineStr"/>
+      <c r="F73" s="2" t="inlineStr"/>
+      <c r="G73" s="2" t="inlineStr"/>
+      <c r="H73" s="2" t="inlineStr"/>
+      <c r="I73" s="2" t="inlineStr"/>
+      <c r="J73" s="2" t="inlineStr"/>
+      <c r="K73" s="2" t="inlineStr"/>
+      <c r="L73" s="2" t="inlineStr"/>
+      <c r="M73" s="2" t="inlineStr"/>
+      <c r="N73" s="2" t="inlineStr"/>
+      <c r="O73" s="2" t="inlineStr">
         <is>
           <t>较清楚</t>
         </is>
       </c>
-      <c r="F73" s="2" t="inlineStr">
+      <c r="P73" s="2" t="inlineStr">
         <is>
           <t>bolt.io</t>
         </is>
@@ -2474,12 +3254,22 @@
           <t>Akero Therapeutics</t>
         </is>
       </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F74" s="2" t="inlineStr">
+      <c r="E74" s="2" t="inlineStr"/>
+      <c r="F74" s="2" t="inlineStr"/>
+      <c r="G74" s="2" t="inlineStr"/>
+      <c r="H74" s="2" t="inlineStr"/>
+      <c r="I74" s="2" t="inlineStr"/>
+      <c r="J74" s="2" t="inlineStr"/>
+      <c r="K74" s="2" t="inlineStr"/>
+      <c r="L74" s="2" t="inlineStr"/>
+      <c r="M74" s="2" t="inlineStr"/>
+      <c r="N74" s="2" t="inlineStr"/>
+      <c r="O74" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P74" s="2" t="inlineStr">
         <is>
           <t>venbio.com</t>
         </is>
@@ -2502,12 +3292,22 @@
           <t>Canva</t>
         </is>
       </c>
-      <c r="E75" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F75" s="2" t="inlineStr">
+      <c r="E75" s="2" t="inlineStr"/>
+      <c r="F75" s="2" t="inlineStr"/>
+      <c r="G75" s="2" t="inlineStr"/>
+      <c r="H75" s="2" t="inlineStr"/>
+      <c r="I75" s="2" t="inlineStr"/>
+      <c r="J75" s="2" t="inlineStr"/>
+      <c r="K75" s="2" t="inlineStr"/>
+      <c r="L75" s="2" t="inlineStr"/>
+      <c r="M75" s="2" t="inlineStr"/>
+      <c r="N75" s="2" t="inlineStr"/>
+      <c r="O75" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P75" s="2" t="inlineStr">
         <is>
           <t>felicis.com</t>
         </is>
@@ -2530,12 +3330,22 @@
           <t>Spark Therapeutics</t>
         </is>
       </c>
-      <c r="E76" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
+      <c r="E76" s="2" t="inlineStr"/>
       <c r="F76" s="2" t="inlineStr"/>
+      <c r="G76" s="2" t="inlineStr"/>
+      <c r="H76" s="2" t="inlineStr"/>
+      <c r="I76" s="2" t="inlineStr"/>
+      <c r="J76" s="2" t="inlineStr"/>
+      <c r="K76" s="2" t="inlineStr"/>
+      <c r="L76" s="2" t="inlineStr"/>
+      <c r="M76" s="2" t="inlineStr"/>
+      <c r="N76" s="2" t="inlineStr"/>
+      <c r="O76" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P76" s="2" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
@@ -2554,12 +3364,22 @@
           <t>Alchemy</t>
         </is>
       </c>
-      <c r="E77" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F77" s="2" t="inlineStr">
+      <c r="E77" s="2" t="inlineStr"/>
+      <c r="F77" s="2" t="inlineStr"/>
+      <c r="G77" s="2" t="inlineStr"/>
+      <c r="H77" s="2" t="inlineStr"/>
+      <c r="I77" s="2" t="inlineStr"/>
+      <c r="J77" s="2" t="inlineStr"/>
+      <c r="K77" s="2" t="inlineStr"/>
+      <c r="L77" s="2" t="inlineStr"/>
+      <c r="M77" s="2" t="inlineStr"/>
+      <c r="N77" s="2" t="inlineStr"/>
+      <c r="O77" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P77" s="2" t="inlineStr">
         <is>
           <t>panteracapital.com</t>
         </is>
@@ -2582,12 +3402,22 @@
           <t>Coinbase</t>
         </is>
       </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F78" s="2" t="inlineStr">
+      <c r="E78" s="2" t="inlineStr"/>
+      <c r="F78" s="2" t="inlineStr"/>
+      <c r="G78" s="2" t="inlineStr"/>
+      <c r="H78" s="2" t="inlineStr"/>
+      <c r="I78" s="2" t="inlineStr"/>
+      <c r="J78" s="2" t="inlineStr"/>
+      <c r="K78" s="2" t="inlineStr"/>
+      <c r="L78" s="2" t="inlineStr"/>
+      <c r="M78" s="2" t="inlineStr"/>
+      <c r="N78" s="2" t="inlineStr"/>
+      <c r="O78" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P78" s="2" t="inlineStr">
         <is>
           <t>initialized.com</t>
         </is>
@@ -2610,12 +3440,22 @@
           <t>Sana Biotechnology</t>
         </is>
       </c>
-      <c r="E79" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F79" s="2" t="inlineStr">
+      <c r="E79" s="2" t="inlineStr"/>
+      <c r="F79" s="2" t="inlineStr"/>
+      <c r="G79" s="2" t="inlineStr"/>
+      <c r="H79" s="2" t="inlineStr"/>
+      <c r="I79" s="2" t="inlineStr"/>
+      <c r="J79" s="2" t="inlineStr"/>
+      <c r="K79" s="2" t="inlineStr"/>
+      <c r="L79" s="2" t="inlineStr"/>
+      <c r="M79" s="2" t="inlineStr"/>
+      <c r="N79" s="2" t="inlineStr"/>
+      <c r="O79" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P79" s="2" t="inlineStr">
         <is>
           <t>fprimecapital.com</t>
         </is>
@@ -2638,12 +3478,22 @@
           <t>Oseberg</t>
         </is>
       </c>
-      <c r="E80" s="2" t="inlineStr">
+      <c r="E80" s="2" t="inlineStr"/>
+      <c r="F80" s="2" t="inlineStr"/>
+      <c r="G80" s="2" t="inlineStr"/>
+      <c r="H80" s="2" t="inlineStr"/>
+      <c r="I80" s="2" t="inlineStr"/>
+      <c r="J80" s="2" t="inlineStr"/>
+      <c r="K80" s="2" t="inlineStr"/>
+      <c r="L80" s="2" t="inlineStr"/>
+      <c r="M80" s="2" t="inlineStr"/>
+      <c r="N80" s="2" t="inlineStr"/>
+      <c r="O80" s="2" t="inlineStr">
         <is>
           <t>已核实（f4.fund 列第 79）</t>
         </is>
       </c>
-      <c r="F80" s="2" t="inlineStr"/>
+      <c r="P80" s="2" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
@@ -2662,12 +3512,22 @@
           <t>Snowflake</t>
         </is>
       </c>
-      <c r="E81" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F81" s="2" t="inlineStr">
+      <c r="E81" s="2" t="inlineStr"/>
+      <c r="F81" s="2" t="inlineStr"/>
+      <c r="G81" s="2" t="inlineStr"/>
+      <c r="H81" s="2" t="inlineStr"/>
+      <c r="I81" s="2" t="inlineStr"/>
+      <c r="J81" s="2" t="inlineStr"/>
+      <c r="K81" s="2" t="inlineStr"/>
+      <c r="L81" s="2" t="inlineStr"/>
+      <c r="M81" s="2" t="inlineStr"/>
+      <c r="N81" s="2" t="inlineStr"/>
+      <c r="O81" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P81" s="2" t="inlineStr">
         <is>
           <t>wing.vc</t>
         </is>
@@ -2690,12 +3550,22 @@
           <t>ServiceTitan</t>
         </is>
       </c>
-      <c r="E82" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
+      <c r="E82" s="2" t="inlineStr"/>
       <c r="F82" s="2" t="inlineStr"/>
+      <c r="G82" s="2" t="inlineStr"/>
+      <c r="H82" s="2" t="inlineStr"/>
+      <c r="I82" s="2" t="inlineStr"/>
+      <c r="J82" s="2" t="inlineStr"/>
+      <c r="K82" s="2" t="inlineStr"/>
+      <c r="L82" s="2" t="inlineStr"/>
+      <c r="M82" s="2" t="inlineStr"/>
+      <c r="N82" s="2" t="inlineStr"/>
+      <c r="O82" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P82" s="2" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
@@ -2714,12 +3584,22 @@
           <t>（看不清）</t>
         </is>
       </c>
-      <c r="E83" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F83" s="2" t="inlineStr">
+      <c r="E83" s="2" t="inlineStr"/>
+      <c r="F83" s="2" t="inlineStr"/>
+      <c r="G83" s="2" t="inlineStr"/>
+      <c r="H83" s="2" t="inlineStr"/>
+      <c r="I83" s="2" t="inlineStr"/>
+      <c r="J83" s="2" t="inlineStr"/>
+      <c r="K83" s="2" t="inlineStr"/>
+      <c r="L83" s="2" t="inlineStr"/>
+      <c r="M83" s="2" t="inlineStr"/>
+      <c r="N83" s="2" t="inlineStr"/>
+      <c r="O83" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P83" s="2" t="inlineStr">
         <is>
           <t>scalevp.com</t>
         </is>
@@ -2742,12 +3622,22 @@
           <t>W 开头的公司（看不清）</t>
         </is>
       </c>
-      <c r="E84" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F84" s="2" t="inlineStr">
+      <c r="E84" s="2" t="inlineStr"/>
+      <c r="F84" s="2" t="inlineStr"/>
+      <c r="G84" s="2" t="inlineStr"/>
+      <c r="H84" s="2" t="inlineStr"/>
+      <c r="I84" s="2" t="inlineStr"/>
+      <c r="J84" s="2" t="inlineStr"/>
+      <c r="K84" s="2" t="inlineStr"/>
+      <c r="L84" s="2" t="inlineStr"/>
+      <c r="M84" s="2" t="inlineStr"/>
+      <c r="N84" s="2" t="inlineStr"/>
+      <c r="O84" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P84" s="2" t="inlineStr">
         <is>
           <t>canaan.com</t>
         </is>
@@ -2770,12 +3660,22 @@
           <t>Fuse</t>
         </is>
       </c>
-      <c r="E85" s="2" t="inlineStr">
+      <c r="E85" s="2" t="inlineStr"/>
+      <c r="F85" s="2" t="inlineStr"/>
+      <c r="G85" s="2" t="inlineStr"/>
+      <c r="H85" s="2" t="inlineStr"/>
+      <c r="I85" s="2" t="inlineStr"/>
+      <c r="J85" s="2" t="inlineStr"/>
+      <c r="K85" s="2" t="inlineStr"/>
+      <c r="L85" s="2" t="inlineStr"/>
+      <c r="M85" s="2" t="inlineStr"/>
+      <c r="N85" s="2" t="inlineStr"/>
+      <c r="O85" s="2" t="inlineStr">
         <is>
           <t>较清楚</t>
         </is>
       </c>
-      <c r="F85" s="2" t="inlineStr">
+      <c r="P85" s="2" t="inlineStr">
         <is>
           <t>multicoin.capital</t>
         </is>
@@ -2798,12 +3698,22 @@
           <t>Etched</t>
         </is>
       </c>
-      <c r="E86" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F86" s="2" t="inlineStr">
+      <c r="E86" s="2" t="inlineStr"/>
+      <c r="F86" s="2" t="inlineStr"/>
+      <c r="G86" s="2" t="inlineStr"/>
+      <c r="H86" s="2" t="inlineStr"/>
+      <c r="I86" s="2" t="inlineStr"/>
+      <c r="J86" s="2" t="inlineStr"/>
+      <c r="K86" s="2" t="inlineStr"/>
+      <c r="L86" s="2" t="inlineStr"/>
+      <c r="M86" s="2" t="inlineStr"/>
+      <c r="N86" s="2" t="inlineStr"/>
+      <c r="O86" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P86" s="2" t="inlineStr">
         <is>
           <t>primary.vc</t>
         </is>
@@ -2826,12 +3736,22 @@
           <t>Coupang</t>
         </is>
       </c>
-      <c r="E87" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
+      <c r="E87" s="2" t="inlineStr"/>
       <c r="F87" s="2" t="inlineStr"/>
+      <c r="G87" s="2" t="inlineStr"/>
+      <c r="H87" s="2" t="inlineStr"/>
+      <c r="I87" s="2" t="inlineStr"/>
+      <c r="J87" s="2" t="inlineStr"/>
+      <c r="K87" s="2" t="inlineStr"/>
+      <c r="L87" s="2" t="inlineStr"/>
+      <c r="M87" s="2" t="inlineStr"/>
+      <c r="N87" s="2" t="inlineStr"/>
+      <c r="O87" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P87" s="2" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
@@ -2850,12 +3770,22 @@
           <t>BillionToOne</t>
         </is>
       </c>
-      <c r="E88" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
+      <c r="E88" s="2" t="inlineStr"/>
       <c r="F88" s="2" t="inlineStr"/>
+      <c r="G88" s="2" t="inlineStr"/>
+      <c r="H88" s="2" t="inlineStr"/>
+      <c r="I88" s="2" t="inlineStr"/>
+      <c r="J88" s="2" t="inlineStr"/>
+      <c r="K88" s="2" t="inlineStr"/>
+      <c r="L88" s="2" t="inlineStr"/>
+      <c r="M88" s="2" t="inlineStr"/>
+      <c r="N88" s="2" t="inlineStr"/>
+      <c r="O88" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P88" s="2" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
@@ -2874,12 +3804,22 @@
           <t>Revolut</t>
         </is>
       </c>
-      <c r="E89" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
+      <c r="E89" s="2" t="inlineStr"/>
       <c r="F89" s="2" t="inlineStr"/>
+      <c r="G89" s="2" t="inlineStr"/>
+      <c r="H89" s="2" t="inlineStr"/>
+      <c r="I89" s="2" t="inlineStr"/>
+      <c r="J89" s="2" t="inlineStr"/>
+      <c r="K89" s="2" t="inlineStr"/>
+      <c r="L89" s="2" t="inlineStr"/>
+      <c r="M89" s="2" t="inlineStr"/>
+      <c r="N89" s="2" t="inlineStr"/>
+      <c r="O89" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P89" s="2" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
@@ -2898,12 +3838,22 @@
           <t>Remote</t>
         </is>
       </c>
-      <c r="E90" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
+      <c r="E90" s="2" t="inlineStr"/>
       <c r="F90" s="2" t="inlineStr"/>
+      <c r="G90" s="2" t="inlineStr"/>
+      <c r="H90" s="2" t="inlineStr"/>
+      <c r="I90" s="2" t="inlineStr"/>
+      <c r="J90" s="2" t="inlineStr"/>
+      <c r="K90" s="2" t="inlineStr"/>
+      <c r="L90" s="2" t="inlineStr"/>
+      <c r="M90" s="2" t="inlineStr"/>
+      <c r="N90" s="2" t="inlineStr"/>
+      <c r="O90" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P90" s="2" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
@@ -2922,12 +3872,22 @@
           <t>Opendoor</t>
         </is>
       </c>
-      <c r="E91" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
+      <c r="E91" s="2" t="inlineStr"/>
       <c r="F91" s="2" t="inlineStr"/>
+      <c r="G91" s="2" t="inlineStr"/>
+      <c r="H91" s="2" t="inlineStr"/>
+      <c r="I91" s="2" t="inlineStr"/>
+      <c r="J91" s="2" t="inlineStr"/>
+      <c r="K91" s="2" t="inlineStr"/>
+      <c r="L91" s="2" t="inlineStr"/>
+      <c r="M91" s="2" t="inlineStr"/>
+      <c r="N91" s="2" t="inlineStr"/>
+      <c r="O91" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P91" s="2" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
@@ -2946,12 +3906,22 @@
           <t>MyoKardia</t>
         </is>
       </c>
-      <c r="E92" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F92" s="2" t="inlineStr">
+      <c r="E92" s="2" t="inlineStr"/>
+      <c r="F92" s="2" t="inlineStr"/>
+      <c r="G92" s="2" t="inlineStr"/>
+      <c r="H92" s="2" t="inlineStr"/>
+      <c r="I92" s="2" t="inlineStr"/>
+      <c r="J92" s="2" t="inlineStr"/>
+      <c r="K92" s="2" t="inlineStr"/>
+      <c r="L92" s="2" t="inlineStr"/>
+      <c r="M92" s="2" t="inlineStr"/>
+      <c r="N92" s="2" t="inlineStr"/>
+      <c r="O92" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P92" s="2" t="inlineStr">
         <is>
           <t>thirdrockventures.com</t>
         </is>
@@ -2974,12 +3944,22 @@
           <t>Pie Insurance</t>
         </is>
       </c>
-      <c r="E93" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F93" s="2" t="inlineStr">
+      <c r="E93" s="2" t="inlineStr"/>
+      <c r="F93" s="2" t="inlineStr"/>
+      <c r="G93" s="2" t="inlineStr"/>
+      <c r="H93" s="2" t="inlineStr"/>
+      <c r="I93" s="2" t="inlineStr"/>
+      <c r="J93" s="2" t="inlineStr"/>
+      <c r="K93" s="2" t="inlineStr"/>
+      <c r="L93" s="2" t="inlineStr"/>
+      <c r="M93" s="2" t="inlineStr"/>
+      <c r="N93" s="2" t="inlineStr"/>
+      <c r="O93" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P93" s="2" t="inlineStr">
         <is>
           <t>greycroft.com</t>
         </is>
@@ -3002,12 +3982,22 @@
           <t>ClickUp</t>
         </is>
       </c>
-      <c r="E94" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F94" s="2" t="inlineStr">
+      <c r="E94" s="2" t="inlineStr"/>
+      <c r="F94" s="2" t="inlineStr"/>
+      <c r="G94" s="2" t="inlineStr"/>
+      <c r="H94" s="2" t="inlineStr"/>
+      <c r="I94" s="2" t="inlineStr"/>
+      <c r="J94" s="2" t="inlineStr"/>
+      <c r="K94" s="2" t="inlineStr"/>
+      <c r="L94" s="2" t="inlineStr"/>
+      <c r="M94" s="2" t="inlineStr"/>
+      <c r="N94" s="2" t="inlineStr"/>
+      <c r="O94" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P94" s="2" t="inlineStr">
         <is>
           <t>craftventures.com</t>
         </is>
@@ -3030,12 +4020,22 @@
           <t>Coupang</t>
         </is>
       </c>
-      <c r="E95" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F95" s="2" t="inlineStr">
+      <c r="E95" s="2" t="inlineStr"/>
+      <c r="F95" s="2" t="inlineStr"/>
+      <c r="G95" s="2" t="inlineStr"/>
+      <c r="H95" s="2" t="inlineStr"/>
+      <c r="I95" s="2" t="inlineStr"/>
+      <c r="J95" s="2" t="inlineStr"/>
+      <c r="K95" s="2" t="inlineStr"/>
+      <c r="L95" s="2" t="inlineStr"/>
+      <c r="M95" s="2" t="inlineStr"/>
+      <c r="N95" s="2" t="inlineStr"/>
+      <c r="O95" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P95" s="2" t="inlineStr">
         <is>
           <t>goodwatercap.com</t>
         </is>
@@ -3058,12 +4058,22 @@
           <t>Move Industries</t>
         </is>
       </c>
-      <c r="E96" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F96" s="2" t="inlineStr">
+      <c r="E96" s="2" t="inlineStr"/>
+      <c r="F96" s="2" t="inlineStr"/>
+      <c r="G96" s="2" t="inlineStr"/>
+      <c r="H96" s="2" t="inlineStr"/>
+      <c r="I96" s="2" t="inlineStr"/>
+      <c r="J96" s="2" t="inlineStr"/>
+      <c r="K96" s="2" t="inlineStr"/>
+      <c r="L96" s="2" t="inlineStr"/>
+      <c r="M96" s="2" t="inlineStr"/>
+      <c r="N96" s="2" t="inlineStr"/>
+      <c r="O96" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P96" s="2" t="inlineStr">
         <is>
           <t>polychain.capital</t>
         </is>
@@ -3086,12 +4096,22 @@
           <t>Instil Bio</t>
         </is>
       </c>
-      <c r="E97" s="2" t="inlineStr">
+      <c r="E97" s="2" t="inlineStr"/>
+      <c r="F97" s="2" t="inlineStr"/>
+      <c r="G97" s="2" t="inlineStr"/>
+      <c r="H97" s="2" t="inlineStr"/>
+      <c r="I97" s="2" t="inlineStr"/>
+      <c r="J97" s="2" t="inlineStr"/>
+      <c r="K97" s="2" t="inlineStr"/>
+      <c r="L97" s="2" t="inlineStr"/>
+      <c r="M97" s="2" t="inlineStr"/>
+      <c r="N97" s="2" t="inlineStr"/>
+      <c r="O97" s="2" t="inlineStr">
         <is>
           <t>较可能（Instil Bio 最大股东，logo 文字吻合；没找到排名原文）</t>
         </is>
       </c>
-      <c r="F97" s="2" t="inlineStr"/>
+      <c r="P97" s="2" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
@@ -3110,12 +4130,22 @@
           <t>Bridge</t>
         </is>
       </c>
-      <c r="E98" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
-      <c r="F98" s="2" t="inlineStr">
+      <c r="E98" s="2" t="inlineStr"/>
+      <c r="F98" s="2" t="inlineStr"/>
+      <c r="G98" s="2" t="inlineStr"/>
+      <c r="H98" s="2" t="inlineStr"/>
+      <c r="I98" s="2" t="inlineStr"/>
+      <c r="J98" s="2" t="inlineStr"/>
+      <c r="K98" s="2" t="inlineStr"/>
+      <c r="L98" s="2" t="inlineStr"/>
+      <c r="M98" s="2" t="inlineStr"/>
+      <c r="N98" s="2" t="inlineStr"/>
+      <c r="O98" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P98" s="2" t="inlineStr">
         <is>
           <t>haun.co</t>
         </is>
@@ -3138,12 +4168,22 @@
           <t>AlphaSense</t>
         </is>
       </c>
-      <c r="E99" s="2" t="inlineStr">
+      <c r="E99" s="2" t="inlineStr"/>
+      <c r="F99" s="2" t="inlineStr"/>
+      <c r="G99" s="2" t="inlineStr"/>
+      <c r="H99" s="2" t="inlineStr"/>
+      <c r="I99" s="2" t="inlineStr"/>
+      <c r="J99" s="2" t="inlineStr"/>
+      <c r="K99" s="2" t="inlineStr"/>
+      <c r="L99" s="2" t="inlineStr"/>
+      <c r="M99" s="2" t="inlineStr"/>
+      <c r="N99" s="2" t="inlineStr"/>
+      <c r="O99" s="2" t="inlineStr">
         <is>
           <t>待确认（领投过 AlphaSense B 轮；没找到排名原文）</t>
         </is>
       </c>
-      <c r="F99" s="2" t="inlineStr"/>
+      <c r="P99" s="2" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
@@ -3162,12 +4202,22 @@
           <t>Poppi</t>
         </is>
       </c>
-      <c r="E100" s="2" t="inlineStr">
+      <c r="E100" s="2" t="inlineStr"/>
+      <c r="F100" s="2" t="inlineStr"/>
+      <c r="G100" s="2" t="inlineStr"/>
+      <c r="H100" s="2" t="inlineStr"/>
+      <c r="I100" s="2" t="inlineStr"/>
+      <c r="J100" s="2" t="inlineStr"/>
+      <c r="K100" s="2" t="inlineStr"/>
+      <c r="L100" s="2" t="inlineStr"/>
+      <c r="M100" s="2" t="inlineStr"/>
+      <c r="N100" s="2" t="inlineStr"/>
+      <c r="O100" s="2" t="inlineStr">
         <is>
           <t>较清楚</t>
         </is>
       </c>
-      <c r="F100" s="2" t="inlineStr"/>
+      <c r="P100" s="2" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
@@ -3186,15 +4236,25 @@
           <t>Metropolis</t>
         </is>
       </c>
-      <c r="E101" s="2" t="inlineStr">
-        <is>
-          <t>清楚</t>
-        </is>
-      </c>
+      <c r="E101" s="2" t="inlineStr"/>
       <c r="F101" s="2" t="inlineStr"/>
+      <c r="G101" s="2" t="inlineStr"/>
+      <c r="H101" s="2" t="inlineStr"/>
+      <c r="I101" s="2" t="inlineStr"/>
+      <c r="J101" s="2" t="inlineStr"/>
+      <c r="K101" s="2" t="inlineStr"/>
+      <c r="L101" s="2" t="inlineStr"/>
+      <c r="M101" s="2" t="inlineStr"/>
+      <c r="N101" s="2" t="inlineStr"/>
+      <c r="O101" s="2" t="inlineStr">
+        <is>
+          <t>清楚</t>
+        </is>
+      </c>
+      <c r="P101" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F101"/>
+  <autoFilter ref="A1:P101"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3205,7 +4265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -3235,6 +4295,13 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>投资阶段：每家投哪些轮次、主力阶段、有没有专门的种子项目（如 Sequoia Arc、a16z speedrun、Greylock Edge）、首笔金额和是否领投，附来源；'适合我们的种子轮'按对 3 周大的 AI 公司种子轮的可能性分 A / B / C。A 档和把握低的条目由第二个调研员复核过。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>SimReal-Top100VC-Apollo导入.csv 收了除'待确认'以外的机构（Company Name, Website 两列），可以在 Apollo 里用 CSV 导入批量查公司；'待确认'的几家可以按括号里的候选名单独搜。</t>
         </is>
       </c>

</xml_diff>